<commit_message>
update VentSpace fix the namelock
</commit_message>
<xml_diff>
--- a/qa/manual/test-cases/Database/Database_testCase.xlsx
+++ b/qa/manual/test-cases/Database/Database_testCase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\freeSpace-main\qa\manual\test-cases\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8316D57D-0740-4956-BD50-EC63B0FCACD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A227BA9-3F94-47EC-9346-663C6EF4CB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="347">
   <si>
     <t>TC ID</t>
   </si>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="C2" s="2">
         <f>COUNTIF('DB Posts'!H2:H100,"Passed")</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D2" s="2">
         <f>COUNTIF('DB Posts'!H2:H100,"Failed")</f>
@@ -1621,11 +1621,11 @@
       </c>
       <c r="E2" s="2" t="str">
         <f t="shared" ref="E2:E9" si="0">IF(B2=0,"0%",TEXT((C2+D2)/B2,"0%"))</f>
-        <v>70%</v>
+        <v>100%</v>
       </c>
       <c r="F2" s="2" t="str">
         <f t="shared" ref="F2:F10" si="1">IF(D2&gt;0,"Blocked",IF(C2&gt;=B2,"Complete","In Progress"))</f>
-        <v>In Progress</v>
+        <v>Complete</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="C3" s="2">
         <f>COUNTIF('DB Comments'!H2:H100,"Passed")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D3" s="2">
         <f>COUNTIF('DB Comments'!H2:H100,"Failed")</f>
@@ -1646,11 +1646,11 @@
       </c>
       <c r="E3" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
       <c r="F3" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>In Progress</v>
+        <v>Complete</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="C10" s="3">
         <f>SUM(C2:C9)</f>
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D10" s="3">
         <f>SUM(D2:D9)</f>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="E10" s="3" t="str">
         <f>TEXT((C10+D10)/B10,"0%")</f>
-        <v>18%</v>
+        <v>38%</v>
       </c>
       <c r="F10" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2598,8 +2598,12 @@
       <c r="F9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="G9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I9" s="7" t="s">
         <v>59</v>
       </c>
@@ -2623,8 +2627,12 @@
       <c r="F10" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I10" s="7" t="s">
         <v>66</v>
       </c>
@@ -2648,8 +2656,12 @@
       <c r="F11" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
+      <c r="G11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I11" s="7" t="s">
         <v>73</v>
       </c>
@@ -2736,8 +2748,12 @@
       <c r="F2" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="G2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I2" s="7" t="s">
         <v>94</v>
       </c>
@@ -2761,8 +2777,12 @@
       <c r="F3" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I3" s="7" t="s">
         <v>101</v>
       </c>
@@ -2786,8 +2806,12 @@
       <c r="F4" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I4" s="7" t="s">
         <v>94</v>
       </c>
@@ -2811,8 +2835,12 @@
       <c r="F5" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="G5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I5" s="7" t="s">
         <v>94</v>
       </c>
@@ -2836,8 +2864,12 @@
       <c r="F6" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
+      <c r="G6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I6" s="7" t="s">
         <v>120</v>
       </c>

</xml_diff>